<commit_message>
Add recoded event data
Instead of 3 variables, we recode events to 2 variables (unexpectedness and outcome importance)
</commit_message>
<xml_diff>
--- a/AnalysisResults/f1_event_impact_summary.xlsx
+++ b/AnalysisResults/f1_event_impact_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,15 +441,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>comment_count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>avg_text_len</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>avg_time_gap</t>
         </is>
@@ -465,13 +470,16 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>84.125</v>
+        <v>752</v>
       </c>
       <c r="D2" t="n">
-        <v>24.0002313777267</v>
+        <v>84.0811170212766</v>
       </c>
       <c r="E2" t="n">
-        <v>2.671627600651064</v>
+        <v>19.27502310174557</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.669721886994039</v>
       </c>
     </row>
     <row r="3">
@@ -484,32 +492,40 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>129.8453608247423</v>
+        <v>97</v>
       </c>
       <c r="D3" t="n">
-        <v>22.27409343799107</v>
+        <v>129.7938144329897</v>
       </c>
       <c r="E3" t="n">
-        <v>1.976235604419905</v>
+        <v>18.05156509061218</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.979685951612877</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ev_resp</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
+          <t>ev_unexp</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Diff(1-0)</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>89.64705882352941</v>
+        <v>97</v>
       </c>
       <c r="D4" t="n">
-        <v>23.90388952814003</v>
+        <v>45.71269741171308</v>
       </c>
       <c r="E4" t="n">
-        <v>2.626741559527576</v>
+        <v>-1.223458011133395</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.6900359353811625</v>
       </c>
     </row>
     <row r="5">
@@ -519,54 +535,133 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>84.58</v>
+        <v>799</v>
       </c>
       <c r="D5" t="n">
-        <v>22.19106653103447</v>
+        <v>89.59949937421777</v>
       </c>
       <c r="E5" t="n">
-        <v>2.039846065115947</v>
+        <v>19.20571183788884</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.625566918189552</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ev_out</t>
+          <t>ev_resp</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>89.40813648293964</v>
+        <v>50</v>
       </c>
       <c r="D6" t="n">
-        <v>24.03959131611585</v>
+        <v>84.58</v>
       </c>
       <c r="E6" t="n">
-        <v>2.670909668094713</v>
+        <v>18.0091085565774</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.036648573850289</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>ev_resp</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Diff(1-0)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-5.019499374217773</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-1.196603281311436</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.5889183443392625</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>ev_out</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>762</v>
+      </c>
+      <c r="D8" t="n">
+        <v>89.35958005249344</v>
+      </c>
+      <c r="E8" t="n">
+        <v>19.3095150641473</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.669952452712387</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ev_out</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="n">
-        <v>88.82758620689656</v>
-      </c>
-      <c r="D7" t="n">
-        <v>21.73094800753256</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1.902593588852404</v>
+      <c r="C9" t="n">
+        <v>87</v>
+      </c>
+      <c r="D9" t="n">
+        <v>88.81609195402299</v>
+      </c>
+      <c r="E9" t="n">
+        <v>17.60883571749206</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.898352038610665</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ev_out</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Diff(1-0)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>87</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.5434880984704478</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-1.700679346655242</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.7716004141017214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>